<commit_message>
Mover config.toml a .streamlit para aplicar tema oscuro
</commit_message>
<xml_diff>
--- a/datos_limpios.xlsx
+++ b/datos_limpios.xlsx
@@ -587,7 +587,7 @@
         <v>22165247</v>
       </c>
       <c r="O2" t="n">
-        <v>1783294046591</v>
+        <v>1783298846824</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>46208.97739109954</v>
+        <v>46209.03294935185</v>
       </c>
       <c r="R2" t="n">
         <v>0.28</v>
@@ -660,7 +660,7 @@
         <v>4165302</v>
       </c>
       <c r="O3" t="n">
-        <v>1783294046592</v>
+        <v>1783298846826</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>46208.97739111111</v>
+        <v>46209.032949375</v>
       </c>
       <c r="R3" t="n">
         <v>0.07000000000000001</v>
@@ -733,7 +733,7 @@
         <v>10011143</v>
       </c>
       <c r="O4" t="n">
-        <v>1783294046593</v>
+        <v>1783298846827</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>46208.97739112269</v>
+        <v>46209.03294938657</v>
       </c>
       <c r="R4" t="n">
         <v>0.51</v>
@@ -806,7 +806,7 @@
         <v>1908301</v>
       </c>
       <c r="O5" t="n">
-        <v>1783294046594</v>
+        <v>1783298846829</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>46208.97739113426</v>
+        <v>46209.03294940972</v>
       </c>
       <c r="R5" t="n">
         <v>1</v>
@@ -879,7 +879,7 @@
         <v>1586011</v>
       </c>
       <c r="O6" t="n">
-        <v>1783294046595</v>
+        <v>1783298846831</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>46208.97739114583</v>
+        <v>46209.03294943287</v>
       </c>
       <c r="R6" t="n">
         <v>0.22</v>
@@ -952,7 +952,7 @@
         <v>1555958</v>
       </c>
       <c r="O7" t="n">
-        <v>1783294046596</v>
+        <v>1783298846832</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>46208.97739115741</v>
+        <v>46209.03294944444</v>
       </c>
       <c r="R7" t="n">
         <v>0.6899999999999999</v>
@@ -1025,7 +1025,7 @@
         <v>463523</v>
       </c>
       <c r="O8" t="n">
-        <v>1783294046597</v>
+        <v>1783298846833</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>46208.97739116898</v>
+        <v>46209.03294945602</v>
       </c>
       <c r="R8" t="n">
         <v>1.03</v>
@@ -1098,7 +1098,7 @@
         <v>1186160</v>
       </c>
       <c r="O9" t="n">
-        <v>1783294046599</v>
+        <v>1783298846834</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>46208.97739119213</v>
+        <v>46209.03294946759</v>
       </c>
       <c r="R9" t="n">
         <v>2.2</v>
@@ -1171,7 +1171,7 @@
         <v>90862</v>
       </c>
       <c r="O10" t="n">
-        <v>1783294046600</v>
+        <v>1783298846835</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>46208.97739120371</v>
+        <v>46209.03294947917</v>
       </c>
       <c r="R10" t="n">
         <v>1.44</v>
@@ -1244,7 +1244,7 @@
         <v>1364199</v>
       </c>
       <c r="O11" t="n">
-        <v>1783294046601</v>
+        <v>1783298846836</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>46208.97739121528</v>
+        <v>46209.03294949074</v>
       </c>
       <c r="R11" t="n">
         <v>1.13</v>
@@ -1317,7 +1317,7 @@
         <v>4263340</v>
       </c>
       <c r="O12" t="n">
-        <v>1783294046603</v>
+        <v>1783298846837</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>46208.97739123843</v>
+        <v>46209.03294950232</v>
       </c>
       <c r="R12" t="n">
         <v>0.92</v>
@@ -1390,7 +1390,7 @@
         <v>1669945</v>
       </c>
       <c r="O13" t="n">
-        <v>1783294046604</v>
+        <v>1783298846838</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
         </is>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>46208.97739125</v>
+        <v>46209.03294951389</v>
       </c>
       <c r="R13" t="n">
         <v>0.8100000000000001</v>
@@ -1463,7 +1463,7 @@
         <v>2606161</v>
       </c>
       <c r="O14" t="n">
-        <v>1783294046605</v>
+        <v>1783298846839</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>46208.97739126157</v>
+        <v>46209.03294952546</v>
       </c>
       <c r="R14" t="n">
         <v>0.55</v>
@@ -1536,7 +1536,7 @@
         <v>133292</v>
       </c>
       <c r="O15" t="n">
-        <v>1783294046606</v>
+        <v>1783298846840</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>46208.97739127315</v>
+        <v>46209.03294953704</v>
       </c>
       <c r="R15" t="n">
         <v>1.94</v>
@@ -1609,7 +1609,7 @@
         <v>2179850</v>
       </c>
       <c r="O16" t="n">
-        <v>1783294046607</v>
+        <v>1783298846841</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>46208.97739128472</v>
+        <v>46209.03294954861</v>
       </c>
       <c r="R16" t="n">
         <v>0.79</v>
@@ -1682,7 +1682,7 @@
         <v>1996315</v>
       </c>
       <c r="O17" t="n">
-        <v>1783294046609</v>
+        <v>1783298846842</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>46208.97739130787</v>
+        <v>46209.03294956018</v>
       </c>
       <c r="R17" t="n">
         <v>0.44</v>
@@ -1755,7 +1755,7 @@
         <v>602707</v>
       </c>
       <c r="O18" t="n">
-        <v>1783294046610</v>
+        <v>1783298846843</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         </is>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>46208.97739131944</v>
+        <v>46209.03294957176</v>
       </c>
       <c r="R18" t="n">
         <v>0.98</v>
@@ -1828,7 +1828,7 @@
         <v>3959997</v>
       </c>
       <c r="O19" t="n">
-        <v>1783294046611</v>
+        <v>1783298846844</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
@@ -1836,7 +1836,7 @@
         </is>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>46208.97739133102</v>
+        <v>46209.03294958334</v>
       </c>
       <c r="R19" t="n">
         <v>0.71</v>
@@ -1901,7 +1901,7 @@
         <v>1370382</v>
       </c>
       <c r="O20" t="n">
-        <v>1783294046612</v>
+        <v>1783298846845</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
@@ -1909,7 +1909,7 @@
         </is>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>46208.9773913426</v>
+        <v>46209.0329495949</v>
       </c>
       <c r="R20" t="n">
         <v>0.52</v>
@@ -1974,7 +1974,7 @@
         <v>1705147</v>
       </c>
       <c r="O21" t="n">
-        <v>1783294046613</v>
+        <v>1783298846848</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>46208.97739135416</v>
+        <v>46209.03294962963</v>
       </c>
       <c r="R21" t="n">
         <v>2.89</v>
@@ -2047,7 +2047,7 @@
         <v>1394355</v>
       </c>
       <c r="O22" t="n">
-        <v>1783294046614</v>
+        <v>1783298846849</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         </is>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>46208.97739136574</v>
+        <v>46209.0329496412</v>
       </c>
       <c r="R22" t="n">
         <v>1.43</v>
@@ -2120,7 +2120,7 @@
         <v>408622</v>
       </c>
       <c r="O23" t="n">
-        <v>1783294046616</v>
+        <v>1783298846850</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>46208.97739138889</v>
+        <v>46209.03294965278</v>
       </c>
       <c r="R23" t="n">
         <v>1.57</v>
@@ -2193,7 +2193,7 @@
         <v>344191</v>
       </c>
       <c r="O24" t="n">
-        <v>1783294046617</v>
+        <v>1783298846851</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>46208.97739140046</v>
+        <v>46209.03294966435</v>
       </c>
       <c r="R24" t="n">
         <v>1.27</v>
@@ -2266,7 +2266,7 @@
         <v>717380</v>
       </c>
       <c r="O25" t="n">
-        <v>1783294046618</v>
+        <v>1783298846852</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>46208.97739141204</v>
+        <v>46209.03294967593</v>
       </c>
       <c r="R25" t="n">
         <v>0.88</v>
@@ -2339,7 +2339,7 @@
         <v>899158</v>
       </c>
       <c r="O26" t="n">
-        <v>1783294046619</v>
+        <v>1783298846853</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>46208.97739142361</v>
+        <v>46209.0329496875</v>
       </c>
       <c r="R26" t="n">
         <v>0.76</v>
@@ -2412,7 +2412,7 @@
         <v>225993</v>
       </c>
       <c r="O27" t="n">
-        <v>1783294046620</v>
+        <v>1783298846855</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>46208.97739143518</v>
+        <v>46209.03294971065</v>
       </c>
       <c r="R27" t="n">
         <v>1.85</v>
@@ -2485,7 +2485,7 @@
         <v>416164</v>
       </c>
       <c r="O28" t="n">
-        <v>1783294046622</v>
+        <v>1783298846856</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>46208.97739145833</v>
+        <v>46209.03294972222</v>
       </c>
       <c r="R28" t="n">
         <v>2.55</v>
@@ -2558,7 +2558,7 @@
         <v>1273936</v>
       </c>
       <c r="O29" t="n">
-        <v>1783294046623</v>
+        <v>1783298846857</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>46208.97739146991</v>
+        <v>46209.0329497338</v>
       </c>
       <c r="R29" t="n">
         <v>0.76</v>
@@ -2631,7 +2631,7 @@
         <v>170173</v>
       </c>
       <c r="O30" t="n">
-        <v>1783294046624</v>
+        <v>1783298846857</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>46208.97739148148</v>
+        <v>46209.0329497338</v>
       </c>
       <c r="R30" t="n">
         <v>3.37</v>
@@ -2704,7 +2704,7 @@
         <v>19910389</v>
       </c>
       <c r="O31" t="n">
-        <v>1783294046625</v>
+        <v>1783298846858</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>46208.97739149306</v>
+        <v>46209.03294974537</v>
       </c>
       <c r="R31" t="n">
         <v>0.22</v>
@@ -2777,7 +2777,7 @@
         <v>1772585</v>
       </c>
       <c r="O32" t="n">
-        <v>1783294046627</v>
+        <v>1783298846859</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>46208.9773915162</v>
+        <v>46209.03294975695</v>
       </c>
       <c r="R32" t="n">
         <v>0.82</v>
@@ -2850,7 +2850,7 @@
         <v>1749083</v>
       </c>
       <c r="O33" t="n">
-        <v>1783294046628</v>
+        <v>1783298846860</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
         </is>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>46208.97739152778</v>
+        <v>46209.03294976852</v>
       </c>
       <c r="R33" t="n">
         <v>0.74</v>
@@ -2923,7 +2923,7 @@
         <v>1193000</v>
       </c>
       <c r="O34" t="n">
-        <v>1783294046629</v>
+        <v>1783298846861</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>46208.97739153935</v>
+        <v>46209.03294978009</v>
       </c>
       <c r="R34" t="n">
         <v>0.23</v>
@@ -2996,7 +2996,7 @@
         <v>200088</v>
       </c>
       <c r="O35" t="n">
-        <v>1783294046630</v>
+        <v>1783298846862</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
@@ -3004,7 +3004,7 @@
         </is>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>46208.97739155093</v>
+        <v>46209.03294979167</v>
       </c>
       <c r="R35" t="n">
         <v>1.2</v>
@@ -3069,7 +3069,7 @@
         <v>1446722</v>
       </c>
       <c r="O36" t="n">
-        <v>1783294046631</v>
+        <v>1783298846863</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>46208.9773915625</v>
+        <v>46209.03294980324</v>
       </c>
       <c r="R36" t="n">
         <v>0.72</v>
@@ -3142,7 +3142,7 @@
         <v>4265272</v>
       </c>
       <c r="O37" t="n">
-        <v>1783294046633</v>
+        <v>1783298846864</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>46208.97739158565</v>
+        <v>46209.03294981481</v>
       </c>
       <c r="R37" t="n">
         <v>0.68</v>
@@ -3215,7 +3215,7 @@
         <v>1268848</v>
       </c>
       <c r="O38" t="n">
-        <v>1783294046634</v>
+        <v>1783298846865</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
         </is>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>46208.97739159723</v>
+        <v>46209.03294982639</v>
       </c>
       <c r="R38" t="n">
         <v>1.15</v>
@@ -3288,7 +3288,7 @@
         <v>363751</v>
       </c>
       <c r="O39" t="n">
-        <v>1783294046635</v>
+        <v>1783298846866</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
@@ -3296,7 +3296,7 @@
         </is>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>46208.97739160879</v>
+        <v>46209.03294983797</v>
       </c>
       <c r="R39" t="n">
         <v>2.41</v>
@@ -3361,7 +3361,7 @@
         <v>752223</v>
       </c>
       <c r="O40" t="n">
-        <v>1783294046638</v>
+        <v>1783298846867</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
@@ -3369,7 +3369,7 @@
         </is>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>46208.97739164352</v>
+        <v>46209.03294984953</v>
       </c>
       <c r="R40" t="n">
         <v>1.25</v>
@@ -3434,7 +3434,7 @@
         <v>6137138</v>
       </c>
       <c r="O41" t="n">
-        <v>1783294046639</v>
+        <v>1783298846868</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
@@ -3442,7 +3442,7 @@
         </is>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>46208.97739165509</v>
+        <v>46209.03294986111</v>
       </c>
       <c r="R41" t="n">
         <v>0.22</v>
@@ -3507,7 +3507,7 @@
         <v>7879860</v>
       </c>
       <c r="O42" t="n">
-        <v>1783294046640</v>
+        <v>1783298846869</v>
       </c>
       <c r="P42" t="inlineStr">
         <is>
@@ -3515,7 +3515,7 @@
         </is>
       </c>
       <c r="Q42" s="2" t="n">
-        <v>46208.97739166667</v>
+        <v>46209.03294987269</v>
       </c>
       <c r="R42" t="n">
         <v>0.2</v>
@@ -3580,7 +3580,7 @@
         <v>338350</v>
       </c>
       <c r="O43" t="n">
-        <v>1783294046640</v>
+        <v>1783298846870</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
@@ -3588,7 +3588,7 @@
         </is>
       </c>
       <c r="Q43" s="2" t="n">
-        <v>46208.97739166667</v>
+        <v>46209.03294988426</v>
       </c>
       <c r="R43" t="n">
         <v>0.65</v>
@@ -3653,7 +3653,7 @@
         <v>300619</v>
       </c>
       <c r="O44" t="n">
-        <v>1783294046641</v>
+        <v>1783298846871</v>
       </c>
       <c r="P44" t="inlineStr">
         <is>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="Q44" s="2" t="n">
-        <v>46208.97739167824</v>
+        <v>46209.03294989583</v>
       </c>
       <c r="R44" t="n">
         <v>2.51</v>
@@ -3726,7 +3726,7 @@
         <v>1930391</v>
       </c>
       <c r="O45" t="n">
-        <v>1783294046642</v>
+        <v>1783298846872</v>
       </c>
       <c r="P45" t="inlineStr">
         <is>
@@ -3734,7 +3734,7 @@
         </is>
       </c>
       <c r="Q45" s="2" t="n">
-        <v>46208.97739168981</v>
+        <v>46209.03294990741</v>
       </c>
       <c r="R45" t="n">
         <v>0.39</v>
@@ -3799,7 +3799,7 @@
         <v>212061</v>
       </c>
       <c r="O46" t="n">
-        <v>1783294046643</v>
+        <v>1783298846872</v>
       </c>
       <c r="P46" t="inlineStr">
         <is>
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="Q46" s="2" t="n">
-        <v>46208.97739170139</v>
+        <v>46209.03294990741</v>
       </c>
       <c r="R46" t="n">
         <v>3.04</v>
@@ -3872,7 +3872,7 @@
         <v>801437</v>
       </c>
       <c r="O47" t="n">
-        <v>1783294046644</v>
+        <v>1783298846873</v>
       </c>
       <c r="P47" t="inlineStr">
         <is>
@@ -3880,7 +3880,7 @@
         </is>
       </c>
       <c r="Q47" s="2" t="n">
-        <v>46208.97739171296</v>
+        <v>46209.03294991898</v>
       </c>
       <c r="R47" t="n">
         <v>1.92</v>
@@ -3945,7 +3945,7 @@
         <v>5271239</v>
       </c>
       <c r="O48" t="n">
-        <v>1783294046645</v>
+        <v>1783298846874</v>
       </c>
       <c r="P48" t="inlineStr">
         <is>
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>46208.97739172454</v>
+        <v>46209.03294993056</v>
       </c>
       <c r="R48" t="n">
         <v>0.48</v>
@@ -4018,7 +4018,7 @@
         <v>575907</v>
       </c>
       <c r="O49" t="n">
-        <v>1783294046646</v>
+        <v>1783298846875</v>
       </c>
       <c r="P49" t="inlineStr">
         <is>
@@ -4026,7 +4026,7 @@
         </is>
       </c>
       <c r="Q49" s="2" t="n">
-        <v>46208.97739173611</v>
+        <v>46209.03294994213</v>
       </c>
       <c r="R49" t="n">
         <v>0.87</v>
@@ -4091,7 +4091,7 @@
         <v>114771</v>
       </c>
       <c r="O50" t="n">
-        <v>1783294046647</v>
+        <v>1783298846877</v>
       </c>
       <c r="P50" t="inlineStr">
         <is>
@@ -4099,7 +4099,7 @@
         </is>
       </c>
       <c r="Q50" s="2" t="n">
-        <v>46208.97739174769</v>
+        <v>46209.03294996528</v>
       </c>
       <c r="R50" t="n">
         <v>1.06</v>
@@ -4164,7 +4164,7 @@
         <v>34792</v>
       </c>
       <c r="O51" t="n">
-        <v>1783294046648</v>
+        <v>1783298846878</v>
       </c>
       <c r="P51" t="inlineStr">
         <is>
@@ -4172,7 +4172,7 @@
         </is>
       </c>
       <c r="Q51" s="2" t="n">
-        <v>46208.97739175926</v>
+        <v>46209.03294997685</v>
       </c>
       <c r="R51" t="n">
         <v>4.77</v>
@@ -4237,7 +4237,7 @@
         <v>1364257</v>
       </c>
       <c r="O52" t="n">
-        <v>1783294046649</v>
+        <v>1783298846879</v>
       </c>
       <c r="P52" t="inlineStr">
         <is>
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="Q52" s="2" t="n">
-        <v>46208.97739177083</v>
+        <v>46209.03294998842</v>
       </c>
       <c r="R52" t="n">
         <v>0.13</v>
@@ -4310,7 +4310,7 @@
         <v>352782</v>
       </c>
       <c r="O53" t="n">
-        <v>1783294046650</v>
+        <v>1783298846880</v>
       </c>
       <c r="P53" t="inlineStr">
         <is>
@@ -4318,7 +4318,7 @@
         </is>
       </c>
       <c r="Q53" s="2" t="n">
-        <v>46208.97739178241</v>
+        <v>46209.03295</v>
       </c>
       <c r="R53" t="n">
         <v>1.27</v>
@@ -4383,7 +4383,7 @@
         <v>110461</v>
       </c>
       <c r="O54" t="n">
-        <v>1783294046794</v>
+        <v>1783298847048</v>
       </c>
       <c r="P54" t="inlineStr">
         <is>
@@ -4391,7 +4391,7 @@
         </is>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>46208.97739344907</v>
+        <v>46209.03295194444</v>
       </c>
       <c r="R54" t="n">
         <v>1.05</v>
@@ -4456,7 +4456,7 @@
         <v>46066</v>
       </c>
       <c r="O55" t="n">
-        <v>1783294046650</v>
+        <v>1783298846881</v>
       </c>
       <c r="P55" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
         </is>
       </c>
       <c r="Q55" s="2" t="n">
-        <v>46208.97739178241</v>
+        <v>46209.03295001158</v>
       </c>
       <c r="R55" t="n">
         <v>1.51</v>
@@ -4529,7 +4529,7 @@
         <v>1766027</v>
       </c>
       <c r="O56" t="n">
-        <v>1783294046651</v>
+        <v>1783298846882</v>
       </c>
       <c r="P56" t="inlineStr">
         <is>
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="Q56" s="2" t="n">
-        <v>46208.97739179398</v>
+        <v>46209.03295002315</v>
       </c>
       <c r="R56" t="n">
         <v>0.19</v>
@@ -4602,7 +4602,7 @@
         <v>162472</v>
       </c>
       <c r="O57" t="n">
-        <v>1783294046652</v>
+        <v>1783298846884</v>
       </c>
       <c r="P57" t="inlineStr">
         <is>
@@ -4610,7 +4610,7 @@
         </is>
       </c>
       <c r="Q57" s="2" t="n">
-        <v>46208.97739180556</v>
+        <v>46209.0329500463</v>
       </c>
       <c r="R57" t="n">
         <v>2.35</v>
@@ -4675,7 +4675,7 @@
         <v>1091164</v>
       </c>
       <c r="O58" t="n">
-        <v>1783294046653</v>
+        <v>1783298846885</v>
       </c>
       <c r="P58" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
         </is>
       </c>
       <c r="Q58" s="2" t="n">
-        <v>46208.97739181713</v>
+        <v>46209.03295005787</v>
       </c>
       <c r="R58" t="n">
         <v>1.94</v>
@@ -4748,7 +4748,7 @@
         <v>580036</v>
       </c>
       <c r="O59" t="n">
-        <v>1783294046654</v>
+        <v>1783298846886</v>
       </c>
       <c r="P59" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
         </is>
       </c>
       <c r="Q59" s="2" t="n">
-        <v>46208.9773918287</v>
+        <v>46209.03295006944</v>
       </c>
       <c r="R59" t="n">
         <v>4.06</v>
@@ -4821,7 +4821,7 @@
         <v>4695724</v>
       </c>
       <c r="O60" t="n">
-        <v>1783294046655</v>
+        <v>1783298846887</v>
       </c>
       <c r="P60" t="inlineStr">
         <is>
@@ -4829,7 +4829,7 @@
         </is>
       </c>
       <c r="Q60" s="2" t="n">
-        <v>46208.97739184028</v>
+        <v>46209.03295008102</v>
       </c>
       <c r="R60" t="n">
         <v>1.16</v>
@@ -4894,7 +4894,7 @@
         <v>7140959</v>
       </c>
       <c r="O61" t="n">
-        <v>1783294046656</v>
+        <v>1783298846888</v>
       </c>
       <c r="P61" t="inlineStr">
         <is>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="Q61" s="2" t="n">
-        <v>46208.97739185185</v>
+        <v>46209.03295009259</v>
       </c>
       <c r="R61" t="n">
         <v>0.31</v>
@@ -4967,7 +4967,7 @@
         <v>1069626</v>
       </c>
       <c r="O62" t="n">
-        <v>1783294046657</v>
+        <v>1783298846889</v>
       </c>
       <c r="P62" t="inlineStr">
         <is>
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="Q62" s="2" t="n">
-        <v>46208.97739186342</v>
+        <v>46209.03295010416</v>
       </c>
       <c r="R62" t="n">
         <v>2.85</v>
@@ -5040,7 +5040,7 @@
         <v>211244</v>
       </c>
       <c r="O63" t="n">
-        <v>1783294046657</v>
+        <v>1783298846890</v>
       </c>
       <c r="P63" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
         </is>
       </c>
       <c r="Q63" s="2" t="n">
-        <v>46208.97739186342</v>
+        <v>46209.03295011574</v>
       </c>
       <c r="R63" t="n">
         <v>1.16</v>
@@ -5113,7 +5113,7 @@
         <v>70569</v>
       </c>
       <c r="O64" t="n">
-        <v>1783294046658</v>
+        <v>1783298846892</v>
       </c>
       <c r="P64" t="inlineStr">
         <is>
@@ -5121,7 +5121,7 @@
         </is>
       </c>
       <c r="Q64" s="2" t="n">
-        <v>46208.977391875</v>
+        <v>46209.03295013889</v>
       </c>
       <c r="R64" t="n">
         <v>1.65</v>
@@ -5186,7 +5186,7 @@
         <v>1611437</v>
       </c>
       <c r="O65" t="n">
-        <v>1783294046659</v>
+        <v>1783298846893</v>
       </c>
       <c r="P65" t="inlineStr">
         <is>
@@ -5194,7 +5194,7 @@
         </is>
       </c>
       <c r="Q65" s="2" t="n">
-        <v>46208.97739188658</v>
+        <v>46209.03295015046</v>
       </c>
       <c r="R65" t="n">
         <v>0.07000000000000001</v>
@@ -5259,7 +5259,7 @@
         <v>677173</v>
       </c>
       <c r="O66" t="n">
-        <v>1783294046660</v>
+        <v>1783298846894</v>
       </c>
       <c r="P66" t="inlineStr">
         <is>
@@ -5267,7 +5267,7 @@
         </is>
       </c>
       <c r="Q66" s="2" t="n">
-        <v>46208.97739189814</v>
+        <v>46209.03295016204</v>
       </c>
       <c r="R66" t="n">
         <v>1.08</v>
@@ -5332,7 +5332,7 @@
         <v>830300</v>
       </c>
       <c r="O67" t="n">
-        <v>1783294046661</v>
+        <v>1783298846896</v>
       </c>
       <c r="P67" t="inlineStr">
         <is>
@@ -5340,7 +5340,7 @@
         </is>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>46208.97739190972</v>
+        <v>46209.03295018519</v>
       </c>
       <c r="R67" t="n">
         <v>0.85</v>
@@ -5405,7 +5405,7 @@
         <v>4410034</v>
       </c>
       <c r="O68" t="n">
-        <v>1783294046662</v>
+        <v>1783298846897</v>
       </c>
       <c r="P68" t="inlineStr">
         <is>
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="Q68" s="2" t="n">
-        <v>46208.9773919213</v>
+        <v>46209.03295019676</v>
       </c>
       <c r="R68" t="n">
         <v>0.96</v>
@@ -5478,7 +5478,7 @@
         <v>5093</v>
       </c>
       <c r="O69" t="n">
-        <v>1783294046663</v>
+        <v>1783298846898</v>
       </c>
       <c r="P69" t="inlineStr">
         <is>
@@ -5486,7 +5486,7 @@
         </is>
       </c>
       <c r="Q69" s="2" t="n">
-        <v>46208.97739193287</v>
+        <v>46209.03295020833</v>
       </c>
       <c r="R69" t="n">
         <v>2.53</v>
@@ -5551,7 +5551,7 @@
         <v>26339</v>
       </c>
       <c r="O70" t="n">
-        <v>1783294046664</v>
+        <v>1783298846899</v>
       </c>
       <c r="P70" t="inlineStr">
         <is>
@@ -5559,7 +5559,7 @@
         </is>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>46208.97739194444</v>
+        <v>46209.03295021991</v>
       </c>
       <c r="R70" t="n">
         <v>1.18</v>
@@ -5624,7 +5624,7 @@
         <v>164744</v>
       </c>
       <c r="O71" t="n">
-        <v>1783294046665</v>
+        <v>1783298846902</v>
       </c>
       <c r="P71" t="inlineStr">
         <is>
@@ -5632,7 +5632,7 @@
         </is>
       </c>
       <c r="Q71" s="2" t="n">
-        <v>46208.97739195602</v>
+        <v>46209.03295025463</v>
       </c>
       <c r="R71" t="n">
         <v>2.15</v>
@@ -5697,7 +5697,7 @@
         <v>40077</v>
       </c>
       <c r="O72" t="n">
-        <v>1783294046666</v>
+        <v>1783298846904</v>
       </c>
       <c r="P72" t="inlineStr">
         <is>
@@ -5705,7 +5705,7 @@
         </is>
       </c>
       <c r="Q72" s="2" t="n">
-        <v>46208.97739196759</v>
+        <v>46209.03295027777</v>
       </c>
       <c r="R72" t="n">
         <v>0.65</v>
@@ -5770,7 +5770,7 @@
         <v>34125</v>
       </c>
       <c r="O73" t="n">
-        <v>1783294046667</v>
+        <v>1783298846905</v>
       </c>
       <c r="P73" t="inlineStr">
         <is>
@@ -5778,7 +5778,7 @@
         </is>
       </c>
       <c r="Q73" s="2" t="n">
-        <v>46208.97739197917</v>
+        <v>46209.03295028935</v>
       </c>
       <c r="R73" t="n">
         <v>3.41</v>
@@ -5843,7 +5843,7 @@
         <v>41437</v>
       </c>
       <c r="O74" t="n">
-        <v>1783294046668</v>
+        <v>1783298846907</v>
       </c>
       <c r="P74" t="inlineStr">
         <is>
@@ -5851,7 +5851,7 @@
         </is>
       </c>
       <c r="Q74" s="2" t="n">
-        <v>46208.97739199074</v>
+        <v>46209.0329503125</v>
       </c>
       <c r="R74" t="n">
         <v>0.96</v>
@@ -5916,7 +5916,7 @@
         <v>2215870</v>
       </c>
       <c r="O75" t="n">
-        <v>1783294046669</v>
+        <v>1783298846909</v>
       </c>
       <c r="P75" t="inlineStr">
         <is>
@@ -5924,7 +5924,7 @@
         </is>
       </c>
       <c r="Q75" s="2" t="n">
-        <v>46208.97739200231</v>
+        <v>46209.03295033565</v>
       </c>
       <c r="R75" t="n">
         <v>0.48</v>
@@ -5989,7 +5989,7 @@
         <v>164845</v>
       </c>
       <c r="O76" t="n">
-        <v>1783294046670</v>
+        <v>1783298846911</v>
       </c>
       <c r="P76" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         </is>
       </c>
       <c r="Q76" s="2" t="n">
-        <v>46208.97739201389</v>
+        <v>46209.03295035879</v>
       </c>
       <c r="R76" t="n">
         <v>0.35</v>
@@ -6062,7 +6062,7 @@
         <v>5780036</v>
       </c>
       <c r="O77" t="n">
-        <v>1783294046672</v>
+        <v>1783298846912</v>
       </c>
       <c r="P77" t="inlineStr">
         <is>
@@ -6070,7 +6070,7 @@
         </is>
       </c>
       <c r="Q77" s="2" t="n">
-        <v>46208.97739203704</v>
+        <v>46209.03295037037</v>
       </c>
       <c r="R77" t="n">
         <v>0.11</v>
@@ -6135,7 +6135,7 @@
         <v>283460</v>
       </c>
       <c r="O78" t="n">
-        <v>1783294046673</v>
+        <v>1783298846914</v>
       </c>
       <c r="P78" t="inlineStr">
         <is>
@@ -6143,7 +6143,7 @@
         </is>
       </c>
       <c r="Q78" s="2" t="n">
-        <v>46208.97739204861</v>
+        <v>46209.03295039352</v>
       </c>
       <c r="R78" t="n">
         <v>1.45</v>
@@ -6208,7 +6208,7 @@
         <v>2346306</v>
       </c>
       <c r="O79" t="n">
-        <v>1783294046674</v>
+        <v>1783298846915</v>
       </c>
       <c r="P79" t="inlineStr">
         <is>
@@ -6216,7 +6216,7 @@
         </is>
       </c>
       <c r="Q79" s="2" t="n">
-        <v>46208.97739206019</v>
+        <v>46209.03295040509</v>
       </c>
       <c r="R79" t="n">
         <v>0.5</v>
@@ -6281,7 +6281,7 @@
         <v>398467</v>
       </c>
       <c r="O80" t="n">
-        <v>1783294046675</v>
+        <v>1783298846917</v>
       </c>
       <c r="P80" t="inlineStr">
         <is>
@@ -6289,7 +6289,7 @@
         </is>
       </c>
       <c r="Q80" s="2" t="n">
-        <v>46208.97739207176</v>
+        <v>46209.03295042824</v>
       </c>
       <c r="R80" t="n">
         <v>2.1</v>
@@ -6354,7 +6354,7 @@
         <v>649295</v>
       </c>
       <c r="O81" t="n">
-        <v>1783294046676</v>
+        <v>1783298846918</v>
       </c>
       <c r="P81" t="inlineStr">
         <is>
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="Q81" s="2" t="n">
-        <v>46208.97739208333</v>
+        <v>46209.03295043982</v>
       </c>
       <c r="R81" t="n">
         <v>2.29</v>
@@ -6427,7 +6427,7 @@
         <v>4092223</v>
       </c>
       <c r="O82" t="n">
-        <v>1783294046677</v>
+        <v>1783298846919</v>
       </c>
       <c r="P82" t="inlineStr">
         <is>
@@ -6435,7 +6435,7 @@
         </is>
       </c>
       <c r="Q82" s="2" t="n">
-        <v>46208.97739209491</v>
+        <v>46209.03295045139</v>
       </c>
       <c r="R82" t="n">
         <v>0.17</v>
@@ -6500,7 +6500,7 @@
         <v>403460</v>
       </c>
       <c r="O83" t="n">
-        <v>1783294046678</v>
+        <v>1783298846921</v>
       </c>
       <c r="P83" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="Q83" s="2" t="n">
-        <v>46208.97739210648</v>
+        <v>46209.03295047454</v>
       </c>
       <c r="R83" t="n">
         <v>2.38</v>
@@ -6573,7 +6573,7 @@
         <v>62198</v>
       </c>
       <c r="O84" t="n">
-        <v>1783294046680</v>
+        <v>1783298846925</v>
       </c>
       <c r="P84" t="inlineStr">
         <is>
@@ -6581,7 +6581,7 @@
         </is>
       </c>
       <c r="Q84" s="2" t="n">
-        <v>46208.97739212963</v>
+        <v>46209.03295052084</v>
       </c>
       <c r="R84" t="n">
         <v>2.11</v>
@@ -6646,7 +6646,7 @@
         <v>78456</v>
       </c>
       <c r="O85" t="n">
-        <v>1783294046681</v>
+        <v>1783298846926</v>
       </c>
       <c r="P85" t="inlineStr">
         <is>
@@ -6654,7 +6654,7 @@
         </is>
       </c>
       <c r="Q85" s="2" t="n">
-        <v>46208.97739214121</v>
+        <v>46209.0329505324</v>
       </c>
       <c r="R85" t="n">
         <v>0.85</v>
@@ -6719,7 +6719,7 @@
         <v>396633</v>
       </c>
       <c r="O86" t="n">
-        <v>1783294046682</v>
+        <v>1783298846927</v>
       </c>
       <c r="P86" t="inlineStr">
         <is>
@@ -6727,7 +6727,7 @@
         </is>
       </c>
       <c r="Q86" s="2" t="n">
-        <v>46208.97739215278</v>
+        <v>46209.03295054398</v>
       </c>
       <c r="R86" t="n">
         <v>2.39</v>
@@ -6792,7 +6792,7 @@
         <v>180062</v>
       </c>
       <c r="O87" t="n">
-        <v>1783294046683</v>
+        <v>1783298846928</v>
       </c>
       <c r="P87" t="inlineStr">
         <is>
@@ -6800,7 +6800,7 @@
         </is>
       </c>
       <c r="Q87" s="2" t="n">
-        <v>46208.97739216435</v>
+        <v>46209.03295055556</v>
       </c>
       <c r="R87" t="n">
         <v>2.2</v>
@@ -6865,7 +6865,7 @@
         <v>442778</v>
       </c>
       <c r="O88" t="n">
-        <v>1783294046684</v>
+        <v>1783298846929</v>
       </c>
       <c r="P88" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="Q88" s="2" t="n">
-        <v>46208.97739217593</v>
+        <v>46209.03295056713</v>
       </c>
       <c r="R88" t="n">
         <v>1.1</v>
@@ -6938,7 +6938,7 @@
         <v>62762</v>
       </c>
       <c r="O89" t="n">
-        <v>1783294046685</v>
+        <v>1783298846930</v>
       </c>
       <c r="P89" t="inlineStr">
         <is>
@@ -6946,7 +6946,7 @@
         </is>
       </c>
       <c r="Q89" s="2" t="n">
-        <v>46208.9773921875</v>
+        <v>46209.0329505787</v>
       </c>
       <c r="R89" t="n">
         <v>1.57</v>
@@ -7011,7 +7011,7 @@
         <v>4888375</v>
       </c>
       <c r="O90" t="n">
-        <v>1783294046686</v>
+        <v>1783298846930</v>
       </c>
       <c r="P90" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         </is>
       </c>
       <c r="Q90" s="2" t="n">
-        <v>46208.97739219907</v>
+        <v>46209.0329505787</v>
       </c>
       <c r="R90" t="n">
         <v>0.73</v>
@@ -7084,7 +7084,7 @@
         <v>2826715</v>
       </c>
       <c r="O91" t="n">
-        <v>1783294046687</v>
+        <v>1783298846931</v>
       </c>
       <c r="P91" t="inlineStr">
         <is>
@@ -7092,7 +7092,7 @@
         </is>
       </c>
       <c r="Q91" s="2" t="n">
-        <v>46208.97739221065</v>
+        <v>46209.03295059028</v>
       </c>
       <c r="R91" t="n">
         <v>0.59</v>
@@ -7157,7 +7157,7 @@
         <v>42818</v>
       </c>
       <c r="O92" t="n">
-        <v>1783294046688</v>
+        <v>1783298846932</v>
       </c>
       <c r="P92" t="inlineStr">
         <is>
@@ -7165,7 +7165,7 @@
         </is>
       </c>
       <c r="Q92" s="2" t="n">
-        <v>46208.97739222222</v>
+        <v>46209.03295060185</v>
       </c>
       <c r="R92" t="n">
         <v>1.8</v>
@@ -7230,7 +7230,7 @@
         <v>7099551</v>
       </c>
       <c r="O93" t="n">
-        <v>1783294046689</v>
+        <v>1783298846933</v>
       </c>
       <c r="P93" t="inlineStr">
         <is>
@@ -7238,7 +7238,7 @@
         </is>
       </c>
       <c r="Q93" s="2" t="n">
-        <v>46208.9773922338</v>
+        <v>46209.03295061343</v>
       </c>
       <c r="R93" t="n">
         <v>0.22</v>
@@ -7303,7 +7303,7 @@
         <v>8890</v>
       </c>
       <c r="O94" t="n">
-        <v>1783294046691</v>
+        <v>1783298846934</v>
       </c>
       <c r="P94" t="inlineStr">
         <is>
@@ -7311,7 +7311,7 @@
         </is>
       </c>
       <c r="Q94" s="2" t="n">
-        <v>46208.97739225694</v>
+        <v>46209.032950625</v>
       </c>
       <c r="R94" t="n">
         <v>1.48</v>
@@ -7376,7 +7376,7 @@
         <v>2072951</v>
       </c>
       <c r="O95" t="n">
-        <v>1783294046692</v>
+        <v>1783298846935</v>
       </c>
       <c r="P95" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
         </is>
       </c>
       <c r="Q95" s="2" t="n">
-        <v>46208.97739226852</v>
+        <v>46209.03295063657</v>
       </c>
       <c r="R95" t="n">
         <v>0.43</v>
@@ -7449,7 +7449,7 @@
         <v>30959</v>
       </c>
       <c r="O96" t="n">
-        <v>1783294046693</v>
+        <v>1783298846936</v>
       </c>
       <c r="P96" t="inlineStr">
         <is>
@@ -7457,7 +7457,7 @@
         </is>
       </c>
       <c r="Q96" s="2" t="n">
-        <v>46208.9773922801</v>
+        <v>46209.03295064815</v>
       </c>
       <c r="R96" t="n">
         <v>3</v>
@@ -7522,7 +7522,7 @@
         <v>64946</v>
       </c>
       <c r="O97" t="n">
-        <v>1783294046694</v>
+        <v>1783298846936</v>
       </c>
       <c r="P97" t="inlineStr">
         <is>
@@ -7530,7 +7530,7 @@
         </is>
       </c>
       <c r="Q97" s="2" t="n">
-        <v>46208.97739229166</v>
+        <v>46209.03295064815</v>
       </c>
       <c r="R97" t="n">
         <v>2.21</v>
@@ -7595,7 +7595,7 @@
         <v>60951</v>
       </c>
       <c r="O98" t="n">
-        <v>1783294046695</v>
+        <v>1783298846937</v>
       </c>
       <c r="P98" t="inlineStr">
         <is>
@@ -7603,7 +7603,7 @@
         </is>
       </c>
       <c r="Q98" s="2" t="n">
-        <v>46208.97739230324</v>
+        <v>46209.03295065972</v>
       </c>
       <c r="R98" t="n">
         <v>0.9399999999999999</v>
@@ -7668,7 +7668,7 @@
         <v>405822</v>
       </c>
       <c r="O99" t="n">
-        <v>1783294046696</v>
+        <v>1783298846938</v>
       </c>
       <c r="P99" t="inlineStr">
         <is>
@@ -7676,7 +7676,7 @@
         </is>
       </c>
       <c r="Q99" s="2" t="n">
-        <v>46208.97739231482</v>
+        <v>46209.0329506713</v>
       </c>
       <c r="R99" t="n">
         <v>1.7</v>
@@ -7741,7 +7741,7 @@
         <v>340182</v>
       </c>
       <c r="O100" t="n">
-        <v>1783294046697</v>
+        <v>1783298846939</v>
       </c>
       <c r="P100" t="inlineStr">
         <is>
@@ -7749,7 +7749,7 @@
         </is>
       </c>
       <c r="Q100" s="2" t="n">
-        <v>46208.97739232639</v>
+        <v>46209.03295068287</v>
       </c>
       <c r="R100" t="n">
         <v>0.39</v>
@@ -7814,7 +7814,7 @@
         <v>0</v>
       </c>
       <c r="O101" t="n">
-        <v>1783294046699</v>
+        <v>1783298846940</v>
       </c>
       <c r="P101" t="inlineStr">
         <is>
@@ -7822,7 +7822,7 @@
         </is>
       </c>
       <c r="Q101" s="2" t="n">
-        <v>46208.97739234954</v>
+        <v>46209.03295069445</v>
       </c>
       <c r="R101" t="n">
         <v>0.82</v>
@@ -7887,7 +7887,7 @@
         <v>885119</v>
       </c>
       <c r="O102" t="n">
-        <v>1783294046701</v>
+        <v>1783298846941</v>
       </c>
       <c r="P102" t="inlineStr">
         <is>
@@ -7895,7 +7895,7 @@
         </is>
       </c>
       <c r="Q102" s="2" t="n">
-        <v>46208.97739237268</v>
+        <v>46209.03295070602</v>
       </c>
       <c r="R102" t="n">
         <v>1.9</v>
@@ -7960,7 +7960,7 @@
         <v>923396</v>
       </c>
       <c r="O103" t="n">
-        <v>1783294046702</v>
+        <v>1783298846943</v>
       </c>
       <c r="P103" t="inlineStr">
         <is>
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="Q103" s="2" t="n">
-        <v>46208.97739238426</v>
+        <v>46209.03295072917</v>
       </c>
       <c r="R103" t="n">
         <v>1.75</v>
@@ -8033,7 +8033,7 @@
         <v>1397453</v>
       </c>
       <c r="O104" t="n">
-        <v>1783294046703</v>
+        <v>1783298846944</v>
       </c>
       <c r="P104" t="inlineStr">
         <is>
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="Q104" s="2" t="n">
-        <v>46208.97739239583</v>
+        <v>46209.03295074074</v>
       </c>
       <c r="R104" t="n">
         <v>0.96</v>
@@ -8106,7 +8106,7 @@
         <v>739866</v>
       </c>
       <c r="O105" t="n">
-        <v>1783294046704</v>
+        <v>1783298846945</v>
       </c>
       <c r="P105" t="inlineStr">
         <is>
@@ -8114,7 +8114,7 @@
         </is>
       </c>
       <c r="Q105" s="2" t="n">
-        <v>46208.97739240741</v>
+        <v>46209.03295075231</v>
       </c>
       <c r="R105" t="n">
         <v>1.28</v>
@@ -8179,7 +8179,7 @@
         <v>18210</v>
       </c>
       <c r="O106" t="n">
-        <v>1783294046705</v>
+        <v>1783298846946</v>
       </c>
       <c r="P106" t="inlineStr">
         <is>
@@ -8187,7 +8187,7 @@
         </is>
       </c>
       <c r="Q106" s="2" t="n">
-        <v>46208.97739241898</v>
+        <v>46209.03295076389</v>
       </c>
       <c r="R106" t="n">
         <v>2.08</v>
@@ -8252,7 +8252,7 @@
         <v>707482</v>
       </c>
       <c r="O107" t="n">
-        <v>1783294046706</v>
+        <v>1783298846946</v>
       </c>
       <c r="P107" t="inlineStr">
         <is>
@@ -8260,7 +8260,7 @@
         </is>
       </c>
       <c r="Q107" s="2" t="n">
-        <v>46208.97739243056</v>
+        <v>46209.03295076389</v>
       </c>
       <c r="R107" t="n">
         <v>0.65</v>
@@ -8325,7 +8325,7 @@
         <v>12240</v>
       </c>
       <c r="O108" t="n">
-        <v>1783294046707</v>
+        <v>1783298846947</v>
       </c>
       <c r="P108" t="inlineStr">
         <is>
@@ -8333,7 +8333,7 @@
         </is>
       </c>
       <c r="Q108" s="2" t="n">
-        <v>46208.97739244213</v>
+        <v>46209.03295077546</v>
       </c>
       <c r="R108" t="n">
         <v>7.89</v>
@@ -8398,7 +8398,7 @@
         <v>206030</v>
       </c>
       <c r="O109" t="n">
-        <v>1783294046708</v>
+        <v>1783298846949</v>
       </c>
       <c r="P109" t="inlineStr">
         <is>
@@ -8406,7 +8406,7 @@
         </is>
       </c>
       <c r="Q109" s="2" t="n">
-        <v>46208.9773924537</v>
+        <v>46209.03295079861</v>
       </c>
       <c r="R109" t="n">
         <v>1.56</v>
@@ -8471,7 +8471,7 @@
         <v>2923739</v>
       </c>
       <c r="O110" t="n">
-        <v>1783294046709</v>
+        <v>1783298846949</v>
       </c>
       <c r="P110" t="inlineStr">
         <is>
@@ -8479,7 +8479,7 @@
         </is>
       </c>
       <c r="Q110" s="2" t="n">
-        <v>46208.97739246528</v>
+        <v>46209.03295079861</v>
       </c>
       <c r="R110" t="n">
         <v>0.03</v>
@@ -8544,7 +8544,7 @@
         <v>7553</v>
       </c>
       <c r="O111" t="n">
-        <v>1783294046710</v>
+        <v>1783298846950</v>
       </c>
       <c r="P111" t="inlineStr">
         <is>
@@ -8552,7 +8552,7 @@
         </is>
       </c>
       <c r="Q111" s="2" t="n">
-        <v>46208.97739247685</v>
+        <v>46209.03295081019</v>
       </c>
       <c r="R111" t="n">
         <v>5.48</v>
@@ -8617,7 +8617,7 @@
         <v>27386</v>
       </c>
       <c r="O112" t="n">
-        <v>1783294046711</v>
+        <v>1783298846952</v>
       </c>
       <c r="P112" t="inlineStr">
         <is>
@@ -8625,7 +8625,7 @@
         </is>
       </c>
       <c r="Q112" s="2" t="n">
-        <v>46208.97739248843</v>
+        <v>46209.03295083333</v>
       </c>
       <c r="R112" t="n">
         <v>0.07000000000000001</v>
@@ -8690,7 +8690,7 @@
         <v>0</v>
       </c>
       <c r="O113" t="n">
-        <v>1783294046711</v>
+        <v>1783298846953</v>
       </c>
       <c r="P113" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
         </is>
       </c>
       <c r="Q113" s="2" t="n">
-        <v>46208.97739248843</v>
+        <v>46209.03295084491</v>
       </c>
       <c r="R113" t="n">
         <v>0.34</v>
@@ -8763,7 +8763,7 @@
         <v>695641</v>
       </c>
       <c r="O114" t="n">
-        <v>1783294046712</v>
+        <v>1783298846954</v>
       </c>
       <c r="P114" t="inlineStr">
         <is>
@@ -8771,7 +8771,7 @@
         </is>
       </c>
       <c r="Q114" s="2" t="n">
-        <v>46208.9773925</v>
+        <v>46209.03295085648</v>
       </c>
       <c r="R114" t="n">
         <v>0.63</v>
@@ -8836,7 +8836,7 @@
         <v>3225256</v>
       </c>
       <c r="O115" t="n">
-        <v>1783294046713</v>
+        <v>1783298846955</v>
       </c>
       <c r="P115" t="inlineStr">
         <is>
@@ -8844,7 +8844,7 @@
         </is>
       </c>
       <c r="Q115" s="2" t="n">
-        <v>46208.97739251157</v>
+        <v>46209.03295086806</v>
       </c>
       <c r="R115" t="n">
         <v>0.34</v>
@@ -8909,7 +8909,7 @@
         <v>26813</v>
       </c>
       <c r="O116" t="n">
-        <v>1783294046714</v>
+        <v>1783298846956</v>
       </c>
       <c r="P116" t="inlineStr">
         <is>
@@ -8917,7 +8917,7 @@
         </is>
       </c>
       <c r="Q116" s="2" t="n">
-        <v>46208.97739252315</v>
+        <v>46209.03295087963</v>
       </c>
       <c r="R116" t="n">
         <v>1.43</v>
@@ -8982,7 +8982,7 @@
         <v>3000640</v>
       </c>
       <c r="O117" t="n">
-        <v>1783294046715</v>
+        <v>1783298846957</v>
       </c>
       <c r="P117" t="inlineStr">
         <is>
@@ -8990,7 +8990,7 @@
         </is>
       </c>
       <c r="Q117" s="2" t="n">
-        <v>46208.97739253473</v>
+        <v>46209.0329508912</v>
       </c>
       <c r="R117" t="n">
         <v>0.64</v>
@@ -9055,7 +9055,7 @@
         <v>1653068</v>
       </c>
       <c r="O118" t="n">
-        <v>1783294046716</v>
+        <v>1783298846958</v>
       </c>
       <c r="P118" t="inlineStr">
         <is>
@@ -9063,7 +9063,7 @@
         </is>
       </c>
       <c r="Q118" s="2" t="n">
-        <v>46208.97739254629</v>
+        <v>46209.03295090278</v>
       </c>
       <c r="R118" t="n">
         <v>0.66</v>
@@ -9128,7 +9128,7 @@
         <v>0</v>
       </c>
       <c r="O119" t="n">
-        <v>1783294046717</v>
+        <v>1783298846959</v>
       </c>
       <c r="P119" t="inlineStr">
         <is>
@@ -9136,7 +9136,7 @@
         </is>
       </c>
       <c r="Q119" s="2" t="n">
-        <v>46208.97739255787</v>
+        <v>46209.03295091435</v>
       </c>
       <c r="R119" t="n">
         <v>1.96</v>
@@ -9201,7 +9201,7 @@
         <v>281374</v>
       </c>
       <c r="O120" t="n">
-        <v>1783294046718</v>
+        <v>1783298846961</v>
       </c>
       <c r="P120" t="inlineStr">
         <is>
@@ -9209,7 +9209,7 @@
         </is>
       </c>
       <c r="Q120" s="2" t="n">
-        <v>46208.97739256945</v>
+        <v>46209.0329509375</v>
       </c>
       <c r="R120" t="n">
         <v>2.44</v>
@@ -9274,7 +9274,7 @@
         <v>618038</v>
       </c>
       <c r="O121" t="n">
-        <v>1783294046718</v>
+        <v>1783298846962</v>
       </c>
       <c r="P121" t="inlineStr">
         <is>
@@ -9282,7 +9282,7 @@
         </is>
       </c>
       <c r="Q121" s="2" t="n">
-        <v>46208.97739256945</v>
+        <v>46209.03295094908</v>
       </c>
       <c r="R121" t="n">
         <v>0.45</v>
@@ -9347,7 +9347,7 @@
         <v>93908</v>
       </c>
       <c r="O122" t="n">
-        <v>1783294046719</v>
+        <v>1783298846963</v>
       </c>
       <c r="P122" t="inlineStr">
         <is>
@@ -9355,7 +9355,7 @@
         </is>
       </c>
       <c r="Q122" s="2" t="n">
-        <v>46208.97739258102</v>
+        <v>46209.03295096065</v>
       </c>
       <c r="R122" t="n">
         <v>0.73</v>
@@ -9420,7 +9420,7 @@
         <v>47607</v>
       </c>
       <c r="O123" t="n">
-        <v>1783294046720</v>
+        <v>1783298846964</v>
       </c>
       <c r="P123" t="inlineStr">
         <is>
@@ -9428,7 +9428,7 @@
         </is>
       </c>
       <c r="Q123" s="2" t="n">
-        <v>46208.97739259259</v>
+        <v>46209.03295097222</v>
       </c>
       <c r="R123" t="n">
         <v>1.21</v>
@@ -9493,7 +9493,7 @@
         <v>643767</v>
       </c>
       <c r="O124" t="n">
-        <v>1783294046721</v>
+        <v>1783298846965</v>
       </c>
       <c r="P124" t="inlineStr">
         <is>
@@ -9501,7 +9501,7 @@
         </is>
       </c>
       <c r="Q124" s="2" t="n">
-        <v>46208.97739260417</v>
+        <v>46209.0329509838</v>
       </c>
       <c r="R124" t="n">
         <v>2.22</v>
@@ -9566,7 +9566,7 @@
         <v>1758422</v>
       </c>
       <c r="O125" t="n">
-        <v>1783294046722</v>
+        <v>1783298846967</v>
       </c>
       <c r="P125" t="inlineStr">
         <is>
@@ -9574,7 +9574,7 @@
         </is>
       </c>
       <c r="Q125" s="2" t="n">
-        <v>46208.97739261574</v>
+        <v>46209.03295100694</v>
       </c>
       <c r="R125" t="n">
         <v>0.31</v>
@@ -9639,7 +9639,7 @@
         <v>198199</v>
       </c>
       <c r="O126" t="n">
-        <v>1783294046723</v>
+        <v>1783298846968</v>
       </c>
       <c r="P126" t="inlineStr">
         <is>
@@ -9647,7 +9647,7 @@
         </is>
       </c>
       <c r="Q126" s="2" t="n">
-        <v>46208.97739262731</v>
+        <v>46209.03295101852</v>
       </c>
       <c r="R126" t="n">
         <v>2</v>
@@ -9712,7 +9712,7 @@
         <v>11337</v>
       </c>
       <c r="O127" t="n">
-        <v>1783294046724</v>
+        <v>1783298846970</v>
       </c>
       <c r="P127" t="inlineStr">
         <is>
@@ -9720,7 +9720,7 @@
         </is>
       </c>
       <c r="Q127" s="2" t="n">
-        <v>46208.97739263889</v>
+        <v>46209.03295104166</v>
       </c>
       <c r="R127" t="n">
         <v>2.48</v>
@@ -9785,7 +9785,7 @@
         <v>15802409</v>
       </c>
       <c r="O128" t="n">
-        <v>1783294046725</v>
+        <v>1783298846971</v>
       </c>
       <c r="P128" t="inlineStr">
         <is>
@@ -9793,7 +9793,7 @@
         </is>
       </c>
       <c r="Q128" s="2" t="n">
-        <v>46208.97739265046</v>
+        <v>46209.03295105324</v>
       </c>
       <c r="R128" t="n">
         <v>0.08</v>
@@ -9858,7 +9858,7 @@
         <v>37483</v>
       </c>
       <c r="O129" t="n">
-        <v>1783294046726</v>
+        <v>1783298846972</v>
       </c>
       <c r="P129" t="inlineStr">
         <is>
@@ -9866,7 +9866,7 @@
         </is>
       </c>
       <c r="Q129" s="2" t="n">
-        <v>46208.97739266204</v>
+        <v>46209.03295106482</v>
       </c>
       <c r="R129" t="n">
         <v>2.24</v>
@@ -9931,7 +9931,7 @@
         <v>3311280</v>
       </c>
       <c r="O130" t="n">
-        <v>1783294046727</v>
+        <v>1783298846973</v>
       </c>
       <c r="P130" t="inlineStr">
         <is>
@@ -9939,7 +9939,7 @@
         </is>
       </c>
       <c r="Q130" s="2" t="n">
-        <v>46208.97739267361</v>
+        <v>46209.03295107639</v>
       </c>
       <c r="R130" t="n">
         <v>0.12</v>
@@ -10004,7 +10004,7 @@
         <v>1139752</v>
       </c>
       <c r="O131" t="n">
-        <v>1783294046728</v>
+        <v>1783298846975</v>
       </c>
       <c r="P131" t="inlineStr">
         <is>
@@ -10012,7 +10012,7 @@
         </is>
       </c>
       <c r="Q131" s="2" t="n">
-        <v>46208.97739268518</v>
+        <v>46209.03295109954</v>
       </c>
       <c r="R131" t="n">
         <v>1.36</v>
@@ -10077,7 +10077,7 @@
         <v>47268</v>
       </c>
       <c r="O132" t="n">
-        <v>1783294046729</v>
+        <v>1783298846977</v>
       </c>
       <c r="P132" t="inlineStr">
         <is>
@@ -10085,7 +10085,7 @@
         </is>
       </c>
       <c r="Q132" s="2" t="n">
-        <v>46208.97739269676</v>
+        <v>46209.03295112269</v>
       </c>
       <c r="R132" t="n">
         <v>0.58</v>
@@ -10150,7 +10150,7 @@
         <v>11760</v>
       </c>
       <c r="O133" t="n">
-        <v>1783294046730</v>
+        <v>1783298846978</v>
       </c>
       <c r="P133" t="inlineStr">
         <is>
@@ -10158,7 +10158,7 @@
         </is>
       </c>
       <c r="Q133" s="2" t="n">
-        <v>46208.97739270833</v>
+        <v>46209.03295113426</v>
       </c>
       <c r="R133" t="n">
         <v>0.44</v>
@@ -10223,7 +10223,7 @@
         <v>23778</v>
       </c>
       <c r="O134" t="n">
-        <v>1783294046730</v>
+        <v>1783298846979</v>
       </c>
       <c r="P134" t="inlineStr">
         <is>
@@ -10231,7 +10231,7 @@
         </is>
       </c>
       <c r="Q134" s="2" t="n">
-        <v>46208.97739270833</v>
+        <v>46209.03295114583</v>
       </c>
       <c r="R134" t="n">
         <v>4.98</v>
@@ -10296,7 +10296,7 @@
         <v>701598</v>
       </c>
       <c r="O135" t="n">
-        <v>1783294046731</v>
+        <v>1783298846980</v>
       </c>
       <c r="P135" t="inlineStr">
         <is>
@@ -10304,7 +10304,7 @@
         </is>
       </c>
       <c r="Q135" s="2" t="n">
-        <v>46208.97739271991</v>
+        <v>46209.03295115741</v>
       </c>
       <c r="R135" t="n">
         <v>0.24</v>
@@ -10369,7 +10369,7 @@
         <v>5775414</v>
       </c>
       <c r="O136" t="n">
-        <v>1783294046732</v>
+        <v>1783298846981</v>
       </c>
       <c r="P136" t="inlineStr">
         <is>
@@ -10377,7 +10377,7 @@
         </is>
       </c>
       <c r="Q136" s="2" t="n">
-        <v>46208.97739273148</v>
+        <v>46209.03295116898</v>
       </c>
       <c r="R136" t="n">
         <v>0.49</v>
@@ -10442,7 +10442,7 @@
         <v>0</v>
       </c>
       <c r="O137" t="n">
-        <v>1783294046733</v>
+        <v>1783298846983</v>
       </c>
       <c r="P137" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
         </is>
       </c>
       <c r="Q137" s="2" t="n">
-        <v>46208.97739274306</v>
+        <v>46209.03295119213</v>
       </c>
       <c r="R137" t="n">
         <v>0.77</v>
@@ -10515,7 +10515,7 @@
         <v>59991</v>
       </c>
       <c r="O138" t="n">
-        <v>1783294046734</v>
+        <v>1783298846984</v>
       </c>
       <c r="P138" t="inlineStr">
         <is>
@@ -10523,7 +10523,7 @@
         </is>
       </c>
       <c r="Q138" s="2" t="n">
-        <v>46208.97739275463</v>
+        <v>46209.03295120371</v>
       </c>
       <c r="R138" t="n">
         <v>1.52</v>
@@ -10588,7 +10588,7 @@
         <v>203391</v>
       </c>
       <c r="O139" t="n">
-        <v>1783294046735</v>
+        <v>1783298846985</v>
       </c>
       <c r="P139" t="inlineStr">
         <is>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="Q139" s="2" t="n">
-        <v>46208.9773927662</v>
+        <v>46209.03295121527</v>
       </c>
       <c r="R139" t="n">
         <v>0.59</v>
@@ -10661,7 +10661,7 @@
         <v>11265</v>
       </c>
       <c r="O140" t="n">
-        <v>1783294046736</v>
+        <v>1783298846986</v>
       </c>
       <c r="P140" t="inlineStr">
         <is>
@@ -10669,7 +10669,7 @@
         </is>
       </c>
       <c r="Q140" s="2" t="n">
-        <v>46208.97739277778</v>
+        <v>46209.03295122685</v>
       </c>
       <c r="R140" t="n">
         <v>1.81</v>
@@ -10734,7 +10734,7 @@
         <v>2929559</v>
       </c>
       <c r="O141" t="n">
-        <v>1783294046737</v>
+        <v>1783298846987</v>
       </c>
       <c r="P141" t="inlineStr">
         <is>
@@ -10742,7 +10742,7 @@
         </is>
       </c>
       <c r="Q141" s="2" t="n">
-        <v>46208.97739278935</v>
+        <v>46209.03295123843</v>
       </c>
       <c r="R141" t="n">
         <v>0.44</v>
@@ -10807,7 +10807,7 @@
         <v>15852213</v>
       </c>
       <c r="O142" t="n">
-        <v>1783294046737</v>
+        <v>1783298846988</v>
       </c>
       <c r="P142" t="inlineStr">
         <is>
@@ -10815,7 +10815,7 @@
         </is>
       </c>
       <c r="Q142" s="2" t="n">
-        <v>46208.97739278935</v>
+        <v>46209.03295125</v>
       </c>
       <c r="R142" t="n">
         <v>0.55</v>
@@ -10880,7 +10880,7 @@
         <v>1612523</v>
       </c>
       <c r="O143" t="n">
-        <v>1783294046738</v>
+        <v>1783298846990</v>
       </c>
       <c r="P143" t="inlineStr">
         <is>
@@ -10888,7 +10888,7 @@
         </is>
       </c>
       <c r="Q143" s="2" t="n">
-        <v>46208.97739280092</v>
+        <v>46209.03295127315</v>
       </c>
       <c r="R143" t="n">
         <v>1.21</v>
@@ -10953,7 +10953,7 @@
         <v>16622128</v>
       </c>
       <c r="O144" t="n">
-        <v>1783294046739</v>
+        <v>1783298846993</v>
       </c>
       <c r="P144" t="inlineStr">
         <is>
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="Q144" s="2" t="n">
-        <v>46208.9773928125</v>
+        <v>46209.03295130787</v>
       </c>
       <c r="R144" t="n">
         <v>0.87</v>
@@ -11026,7 +11026,7 @@
         <v>35313</v>
       </c>
       <c r="O145" t="n">
-        <v>1783294046740</v>
+        <v>1783298846993</v>
       </c>
       <c r="P145" t="inlineStr">
         <is>
@@ -11034,7 +11034,7 @@
         </is>
       </c>
       <c r="Q145" s="2" t="n">
-        <v>46208.97739282408</v>
+        <v>46209.03295130787</v>
       </c>
       <c r="R145" t="n">
         <v>0.78</v>
@@ -11099,7 +11099,7 @@
         <v>0</v>
       </c>
       <c r="O146" t="n">
-        <v>1783294046741</v>
+        <v>1783298846994</v>
       </c>
       <c r="P146" t="inlineStr">
         <is>
@@ -11107,7 +11107,7 @@
         </is>
       </c>
       <c r="Q146" s="2" t="n">
-        <v>46208.97739283565</v>
+        <v>46209.03295131944</v>
       </c>
       <c r="R146" t="n">
         <v>1.22</v>
@@ -11172,7 +11172,7 @@
         <v>0</v>
       </c>
       <c r="O147" t="n">
-        <v>1783294046742</v>
+        <v>1783298846996</v>
       </c>
       <c r="P147" t="inlineStr">
         <is>
@@ -11180,7 +11180,7 @@
         </is>
       </c>
       <c r="Q147" s="2" t="n">
-        <v>46208.97739284722</v>
+        <v>46209.03295134259</v>
       </c>
       <c r="R147" t="n">
         <v>0.7</v>
@@ -11245,7 +11245,7 @@
         <v>244342</v>
       </c>
       <c r="O148" t="n">
-        <v>1783294046743</v>
+        <v>1783298846998</v>
       </c>
       <c r="P148" t="inlineStr">
         <is>
@@ -11253,7 +11253,7 @@
         </is>
       </c>
       <c r="Q148" s="2" t="n">
-        <v>46208.9773928588</v>
+        <v>46209.03295136574</v>
       </c>
       <c r="R148" t="n">
         <v>1.06</v>
@@ -11318,7 +11318,7 @@
         <v>1976875</v>
       </c>
       <c r="O149" t="n">
-        <v>1783294046744</v>
+        <v>1783298847000</v>
       </c>
       <c r="P149" t="inlineStr">
         <is>
@@ -11326,7 +11326,7 @@
         </is>
       </c>
       <c r="Q149" s="2" t="n">
-        <v>46208.97739287037</v>
+        <v>46209.03295138889</v>
       </c>
       <c r="R149" t="n">
         <v>0.39</v>
@@ -11391,7 +11391,7 @@
         <v>926612</v>
       </c>
       <c r="O150" t="n">
-        <v>1783294046745</v>
+        <v>1783298847002</v>
       </c>
       <c r="P150" t="inlineStr">
         <is>
@@ -11399,7 +11399,7 @@
         </is>
       </c>
       <c r="Q150" s="2" t="n">
-        <v>46208.97739288194</v>
+        <v>46209.03295141204</v>
       </c>
       <c r="R150" t="n">
         <v>0.18</v>
@@ -11464,7 +11464,7 @@
         <v>4965327</v>
       </c>
       <c r="O151" t="n">
-        <v>1783294046746</v>
+        <v>1783298847003</v>
       </c>
       <c r="P151" t="inlineStr">
         <is>
@@ -11472,7 +11472,7 @@
         </is>
       </c>
       <c r="Q151" s="2" t="n">
-        <v>46208.97739289352</v>
+        <v>46209.03295142361</v>
       </c>
       <c r="R151" t="n">
         <v>0.08</v>
@@ -11537,7 +11537,7 @@
         <v>0</v>
       </c>
       <c r="O152" t="n">
-        <v>1783294046747</v>
+        <v>1783298847006</v>
       </c>
       <c r="P152" t="inlineStr">
         <is>
@@ -11545,7 +11545,7 @@
         </is>
       </c>
       <c r="Q152" s="2" t="n">
-        <v>46208.97739290509</v>
+        <v>46209.03295145834</v>
       </c>
       <c r="R152" t="n">
         <v>0.11</v>
@@ -11610,7 +11610,7 @@
         <v>3170187</v>
       </c>
       <c r="O153" t="n">
-        <v>1783294046748</v>
+        <v>1783298847007</v>
       </c>
       <c r="P153" t="inlineStr">
         <is>
@@ -11618,7 +11618,7 @@
         </is>
       </c>
       <c r="Q153" s="2" t="n">
-        <v>46208.97739291667</v>
+        <v>46209.0329514699</v>
       </c>
       <c r="R153" t="n">
         <v>0.46</v>
@@ -11683,7 +11683,7 @@
         <v>301094</v>
       </c>
       <c r="O154" t="n">
-        <v>1783294046749</v>
+        <v>1783298847009</v>
       </c>
       <c r="P154" t="inlineStr">
         <is>
@@ -11691,7 +11691,7 @@
         </is>
       </c>
       <c r="Q154" s="2" t="n">
-        <v>46208.97739292824</v>
+        <v>46209.03295149306</v>
       </c>
       <c r="R154" t="n">
         <v>1.2</v>
@@ -11756,7 +11756,7 @@
         <v>16205</v>
       </c>
       <c r="O155" t="n">
-        <v>1783294046751</v>
+        <v>1783298847010</v>
       </c>
       <c r="P155" t="inlineStr">
         <is>
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="Q155" s="2" t="n">
-        <v>46208.97739295139</v>
+        <v>46209.03295150463</v>
       </c>
       <c r="R155" t="n">
         <v>0.73</v>
@@ -11829,7 +11829,7 @@
         <v>60851</v>
       </c>
       <c r="O156" t="n">
-        <v>1783294046752</v>
+        <v>1783298847011</v>
       </c>
       <c r="P156" t="inlineStr">
         <is>
@@ -11837,7 +11837,7 @@
         </is>
       </c>
       <c r="Q156" s="2" t="n">
-        <v>46208.97739296297</v>
+        <v>46209.0329515162</v>
       </c>
       <c r="R156" t="n">
         <v>2.95</v>
@@ -11902,7 +11902,7 @@
         <v>2828643</v>
       </c>
       <c r="O157" t="n">
-        <v>1783294046754</v>
+        <v>1783298847012</v>
       </c>
       <c r="P157" t="inlineStr">
         <is>
@@ -11910,7 +11910,7 @@
         </is>
       </c>
       <c r="Q157" s="2" t="n">
-        <v>46208.97739298611</v>
+        <v>46209.03295152778</v>
       </c>
       <c r="R157" t="n">
         <v>0.51</v>
@@ -11975,7 +11975,7 @@
         <v>77606</v>
       </c>
       <c r="O158" t="n">
-        <v>1783294046756</v>
+        <v>1783298847012</v>
       </c>
       <c r="P158" t="inlineStr">
         <is>
@@ -11983,7 +11983,7 @@
         </is>
       </c>
       <c r="Q158" s="2" t="n">
-        <v>46208.97739300926</v>
+        <v>46209.03295152778</v>
       </c>
       <c r="R158" t="n">
         <v>0.12</v>
@@ -12048,7 +12048,7 @@
         <v>2894810</v>
       </c>
       <c r="O159" t="n">
-        <v>1783294046758</v>
+        <v>1783298847014</v>
       </c>
       <c r="P159" t="inlineStr">
         <is>
@@ -12056,7 +12056,7 @@
         </is>
       </c>
       <c r="Q159" s="2" t="n">
-        <v>46208.97739303241</v>
+        <v>46209.03295155093</v>
       </c>
       <c r="R159" t="n">
         <v>0.18</v>
@@ -12121,7 +12121,7 @@
         <v>10579</v>
       </c>
       <c r="O160" t="n">
-        <v>1783294046760</v>
+        <v>1783298847014</v>
       </c>
       <c r="P160" t="inlineStr">
         <is>
@@ -12129,7 +12129,7 @@
         </is>
       </c>
       <c r="Q160" s="2" t="n">
-        <v>46208.97739305555</v>
+        <v>46209.03295155093</v>
       </c>
       <c r="R160" t="n">
         <v>18.07</v>
@@ -12194,7 +12194,7 @@
         <v>1130559</v>
       </c>
       <c r="O161" t="n">
-        <v>1783294046763</v>
+        <v>1783298847015</v>
       </c>
       <c r="P161" t="inlineStr">
         <is>
@@ -12202,7 +12202,7 @@
         </is>
       </c>
       <c r="Q161" s="2" t="n">
-        <v>46208.97739309028</v>
+        <v>46209.0329515625</v>
       </c>
       <c r="R161" t="n">
         <v>0.33</v>
@@ -12267,7 +12267,7 @@
         <v>1411454</v>
       </c>
       <c r="O162" t="n">
-        <v>1783294046764</v>
+        <v>1783298847016</v>
       </c>
       <c r="P162" t="inlineStr">
         <is>
@@ -12275,7 +12275,7 @@
         </is>
       </c>
       <c r="Q162" s="2" t="n">
-        <v>46208.97739310185</v>
+        <v>46209.03295157407</v>
       </c>
       <c r="R162" t="n">
         <v>0.83</v>
@@ -12340,7 +12340,7 @@
         <v>6470</v>
       </c>
       <c r="O163" t="n">
-        <v>1783294046765</v>
+        <v>1783298847017</v>
       </c>
       <c r="P163" t="inlineStr">
         <is>
@@ -12348,7 +12348,7 @@
         </is>
       </c>
       <c r="Q163" s="2" t="n">
-        <v>46208.97739311343</v>
+        <v>46209.03295158565</v>
       </c>
       <c r="R163" t="n">
         <v>1.01</v>
@@ -12413,7 +12413,7 @@
         <v>9759</v>
       </c>
       <c r="O164" t="n">
-        <v>1783294046766</v>
+        <v>1783298847018</v>
       </c>
       <c r="P164" t="inlineStr">
         <is>
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="Q164" s="2" t="n">
-        <v>46208.977393125</v>
+        <v>46209.03295159722</v>
       </c>
       <c r="R164" t="n">
         <v>3.14</v>
@@ -12486,7 +12486,7 @@
         <v>1023720</v>
       </c>
       <c r="O165" t="n">
-        <v>1783294046767</v>
+        <v>1783298847019</v>
       </c>
       <c r="P165" t="inlineStr">
         <is>
@@ -12494,7 +12494,7 @@
         </is>
       </c>
       <c r="Q165" s="2" t="n">
-        <v>46208.97739313657</v>
+        <v>46209.03295160879</v>
       </c>
       <c r="R165" t="n">
         <v>1.28</v>
@@ -12559,7 +12559,7 @@
         <v>70385</v>
       </c>
       <c r="O166" t="n">
-        <v>1783294046768</v>
+        <v>1783298847020</v>
       </c>
       <c r="P166" t="inlineStr">
         <is>
@@ -12567,7 +12567,7 @@
         </is>
       </c>
       <c r="Q166" s="2" t="n">
-        <v>46208.97739314815</v>
+        <v>46209.03295162037</v>
       </c>
       <c r="R166" t="n">
         <v>1.84</v>
@@ -12632,7 +12632,7 @@
         <v>0</v>
       </c>
       <c r="O167" t="n">
-        <v>1783294046769</v>
+        <v>1783298847021</v>
       </c>
       <c r="P167" t="inlineStr">
         <is>
@@ -12640,7 +12640,7 @@
         </is>
       </c>
       <c r="Q167" s="2" t="n">
-        <v>46208.97739315972</v>
+        <v>46209.03295163195</v>
       </c>
       <c r="R167" t="n">
         <v>1.77</v>
@@ -12705,7 +12705,7 @@
         <v>189943</v>
       </c>
       <c r="O168" t="n">
-        <v>1783294046770</v>
+        <v>1783298847022</v>
       </c>
       <c r="P168" t="inlineStr">
         <is>
@@ -12713,7 +12713,7 @@
         </is>
       </c>
       <c r="Q168" s="2" t="n">
-        <v>46208.9773931713</v>
+        <v>46209.03295164352</v>
       </c>
       <c r="R168" t="n">
         <v>1.6</v>
@@ -12778,7 +12778,7 @@
         <v>26356</v>
       </c>
       <c r="O169" t="n">
-        <v>1783294046771</v>
+        <v>1783298847023</v>
       </c>
       <c r="P169" t="inlineStr">
         <is>
@@ -12786,7 +12786,7 @@
         </is>
       </c>
       <c r="Q169" s="2" t="n">
-        <v>46208.97739318287</v>
+        <v>46209.03295165509</v>
       </c>
       <c r="R169" t="n">
         <v>3.65</v>
@@ -12851,7 +12851,7 @@
         <v>31296</v>
       </c>
       <c r="O170" t="n">
-        <v>1783294046772</v>
+        <v>1783298847023</v>
       </c>
       <c r="P170" t="inlineStr">
         <is>
@@ -12859,7 +12859,7 @@
         </is>
       </c>
       <c r="Q170" s="2" t="n">
-        <v>46208.97739319444</v>
+        <v>46209.03295165509</v>
       </c>
       <c r="R170" t="n">
         <v>1.62</v>
@@ -12924,7 +12924,7 @@
         <v>10988</v>
       </c>
       <c r="O171" t="n">
-        <v>1783294046773</v>
+        <v>1783298847024</v>
       </c>
       <c r="P171" t="inlineStr">
         <is>
@@ -12932,7 +12932,7 @@
         </is>
       </c>
       <c r="Q171" s="2" t="n">
-        <v>46208.97739320602</v>
+        <v>46209.03295166667</v>
       </c>
       <c r="R171" t="n">
         <v>2.52</v>
@@ -12997,7 +12997,7 @@
         <v>3508269</v>
       </c>
       <c r="O172" t="n">
-        <v>1783294046774</v>
+        <v>1783298847025</v>
       </c>
       <c r="P172" t="inlineStr">
         <is>
@@ -13005,7 +13005,7 @@
         </is>
       </c>
       <c r="Q172" s="2" t="n">
-        <v>46208.9773932176</v>
+        <v>46209.03295167824</v>
       </c>
       <c r="R172" t="n">
         <v>0.87</v>
@@ -13070,7 +13070,7 @@
         <v>1120596</v>
       </c>
       <c r="O173" t="n">
-        <v>1783294046775</v>
+        <v>1783298847026</v>
       </c>
       <c r="P173" t="inlineStr">
         <is>
@@ -13078,7 +13078,7 @@
         </is>
       </c>
       <c r="Q173" s="2" t="n">
-        <v>46208.97739322916</v>
+        <v>46209.03295168981</v>
       </c>
       <c r="R173" t="n">
         <v>0.03</v>
@@ -13143,7 +13143,7 @@
         <v>130008</v>
       </c>
       <c r="O174" t="n">
-        <v>1783294046775</v>
+        <v>1783298847027</v>
       </c>
       <c r="P174" t="inlineStr">
         <is>
@@ -13151,7 +13151,7 @@
         </is>
       </c>
       <c r="Q174" s="2" t="n">
-        <v>46208.97739322916</v>
+        <v>46209.03295170139</v>
       </c>
       <c r="R174" t="n">
         <v>1.18</v>
@@ -13216,7 +13216,7 @@
         <v>15520193</v>
       </c>
       <c r="O175" t="n">
-        <v>1783294046776</v>
+        <v>1783298847028</v>
       </c>
       <c r="P175" t="inlineStr">
         <is>
@@ -13224,7 +13224,7 @@
         </is>
       </c>
       <c r="Q175" s="2" t="n">
-        <v>46208.97739324074</v>
+        <v>46209.03295171296</v>
       </c>
       <c r="R175" t="n">
         <v>0.59</v>
@@ -13289,7 +13289,7 @@
         <v>2356704</v>
       </c>
       <c r="O176" t="n">
-        <v>1783294046777</v>
+        <v>1783298847029</v>
       </c>
       <c r="P176" t="inlineStr">
         <is>
@@ -13297,7 +13297,7 @@
         </is>
       </c>
       <c r="Q176" s="2" t="n">
-        <v>46208.97739325232</v>
+        <v>46209.03295172453</v>
       </c>
       <c r="R176" t="n">
         <v>0.73</v>
@@ -13362,7 +13362,7 @@
         <v>3917841</v>
       </c>
       <c r="O177" t="n">
-        <v>1783294046778</v>
+        <v>1783298847030</v>
       </c>
       <c r="P177" t="inlineStr">
         <is>
@@ -13370,7 +13370,7 @@
         </is>
       </c>
       <c r="Q177" s="2" t="n">
-        <v>46208.97739326389</v>
+        <v>46209.03295173611</v>
       </c>
       <c r="R177" t="n">
         <v>0.16</v>
@@ -13435,7 +13435,7 @@
         <v>7908095</v>
       </c>
       <c r="O178" t="n">
-        <v>1783294046779</v>
+        <v>1783298847031</v>
       </c>
       <c r="P178" t="inlineStr">
         <is>
@@ -13443,7 +13443,7 @@
         </is>
       </c>
       <c r="Q178" s="2" t="n">
-        <v>46208.97739327546</v>
+        <v>46209.03295174769</v>
       </c>
       <c r="R178" t="n">
         <v>0.11</v>
@@ -13508,7 +13508,7 @@
         <v>1881042</v>
       </c>
       <c r="O179" t="n">
-        <v>1783294046780</v>
+        <v>1783298847032</v>
       </c>
       <c r="P179" t="inlineStr">
         <is>
@@ -13516,7 +13516,7 @@
         </is>
       </c>
       <c r="Q179" s="2" t="n">
-        <v>46208.97739328704</v>
+        <v>46209.03295175926</v>
       </c>
       <c r="R179" t="n">
         <v>0.02</v>
@@ -13581,7 +13581,7 @@
         <v>0</v>
       </c>
       <c r="O180" t="n">
-        <v>1783294046781</v>
+        <v>1783298847033</v>
       </c>
       <c r="P180" t="inlineStr">
         <is>
@@ -13589,7 +13589,7 @@
         </is>
       </c>
       <c r="Q180" s="2" t="n">
-        <v>46208.97739329861</v>
+        <v>46209.03295177083</v>
       </c>
       <c r="R180" t="n">
         <v>0.47</v>
@@ -13654,7 +13654,7 @@
         <v>3373736</v>
       </c>
       <c r="O181" t="n">
-        <v>1783294046782</v>
+        <v>1783298847034</v>
       </c>
       <c r="P181" t="inlineStr">
         <is>
@@ -13662,7 +13662,7 @@
         </is>
       </c>
       <c r="Q181" s="2" t="n">
-        <v>46208.97739331018</v>
+        <v>46209.03295178241</v>
       </c>
       <c r="R181" t="n">
         <v>0.31</v>
@@ -13727,7 +13727,7 @@
         <v>1867419</v>
       </c>
       <c r="O182" t="n">
-        <v>1783294046783</v>
+        <v>1783298847034</v>
       </c>
       <c r="P182" t="inlineStr">
         <is>
@@ -13735,7 +13735,7 @@
         </is>
       </c>
       <c r="Q182" s="2" t="n">
-        <v>46208.97739332176</v>
+        <v>46209.03295178241</v>
       </c>
       <c r="R182" t="n">
         <v>0.23</v>
@@ -13800,7 +13800,7 @@
         <v>4410488</v>
       </c>
       <c r="O183" t="n">
-        <v>1783294046783</v>
+        <v>1783298847035</v>
       </c>
       <c r="P183" t="inlineStr">
         <is>
@@ -13808,7 +13808,7 @@
         </is>
       </c>
       <c r="Q183" s="2" t="n">
-        <v>46208.97739332176</v>
+        <v>46209.03295179398</v>
       </c>
       <c r="R183" t="n">
         <v>0.06</v>
@@ -13873,7 +13873,7 @@
         <v>0</v>
       </c>
       <c r="O184" t="n">
-        <v>1783294046784</v>
+        <v>1783298847036</v>
       </c>
       <c r="P184" t="inlineStr">
         <is>
@@ -13881,7 +13881,7 @@
         </is>
       </c>
       <c r="Q184" s="2" t="n">
-        <v>46208.97739333333</v>
+        <v>46209.03295180556</v>
       </c>
       <c r="R184" t="n">
         <v>0.03</v>
@@ -13946,7 +13946,7 @@
         <v>0</v>
       </c>
       <c r="O185" t="n">
-        <v>1783294046785</v>
+        <v>1783298847037</v>
       </c>
       <c r="P185" t="inlineStr">
         <is>
@@ -13954,7 +13954,7 @@
         </is>
       </c>
       <c r="Q185" s="2" t="n">
-        <v>46208.97739334491</v>
+        <v>46209.03295181713</v>
       </c>
       <c r="R185" t="n">
         <v>0</v>
@@ -14019,7 +14019,7 @@
         <v>2439107</v>
       </c>
       <c r="O186" t="n">
-        <v>1783294046786</v>
+        <v>1783298847038</v>
       </c>
       <c r="P186" t="inlineStr">
         <is>
@@ -14027,7 +14027,7 @@
         </is>
       </c>
       <c r="Q186" s="2" t="n">
-        <v>46208.97739335648</v>
+        <v>46209.0329518287</v>
       </c>
       <c r="R186" t="n">
         <v>0</v>
@@ -14092,7 +14092,7 @@
         <v>3577442</v>
       </c>
       <c r="O187" t="n">
-        <v>1783294046787</v>
+        <v>1783298847039</v>
       </c>
       <c r="P187" t="inlineStr">
         <is>
@@ -14100,7 +14100,7 @@
         </is>
       </c>
       <c r="Q187" s="2" t="n">
-        <v>46208.97739336806</v>
+        <v>46209.03295184028</v>
       </c>
       <c r="R187" t="n">
         <v>0.57</v>
@@ -14165,7 +14165,7 @@
         <v>0</v>
       </c>
       <c r="O188" t="n">
-        <v>1783294046788</v>
+        <v>1783298847040</v>
       </c>
       <c r="P188" t="inlineStr">
         <is>
@@ -14173,7 +14173,7 @@
         </is>
       </c>
       <c r="Q188" s="2" t="n">
-        <v>46208.97739337963</v>
+        <v>46209.03295185185</v>
       </c>
       <c r="R188" t="n">
         <v>0</v>
@@ -14234,11 +14234,11 @@
         <v>0</v>
       </c>
       <c r="O189" t="n">
-        <v>1783294046789</v>
+        <v>1783298847041</v>
       </c>
       <c r="P189" t="inlineStr"/>
       <c r="Q189" s="2" t="n">
-        <v>46208.9773933912</v>
+        <v>46209.03295186342</v>
       </c>
       <c r="R189" t="n">
         <v>1.83</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="O190" t="n">
-        <v>1783294046790</v>
+        <v>1783298847043</v>
       </c>
       <c r="P190" t="inlineStr">
         <is>
@@ -14311,7 +14311,7 @@
         </is>
       </c>
       <c r="Q190" s="2" t="n">
-        <v>46208.97739340278</v>
+        <v>46209.03295188658</v>
       </c>
       <c r="R190" t="n">
         <v>0</v>
@@ -14376,7 +14376,7 @@
         <v>0</v>
       </c>
       <c r="O191" t="n">
-        <v>1783294046791</v>
+        <v>1783298847044</v>
       </c>
       <c r="P191" t="inlineStr">
         <is>
@@ -14384,7 +14384,7 @@
         </is>
       </c>
       <c r="Q191" s="2" t="n">
-        <v>46208.97739341435</v>
+        <v>46209.03295189815</v>
       </c>
       <c r="R191" t="n">
         <v>0</v>
@@ -14449,7 +14449,7 @@
         <v>0</v>
       </c>
       <c r="O192" t="n">
-        <v>1783294046792</v>
+        <v>1783298847045</v>
       </c>
       <c r="P192" t="inlineStr">
         <is>
@@ -14457,7 +14457,7 @@
         </is>
       </c>
       <c r="Q192" s="2" t="n">
-        <v>46208.97739342593</v>
+        <v>46209.03295190972</v>
       </c>
       <c r="R192" t="n">
         <v>10</v>
@@ -14518,11 +14518,11 @@
         <v>0</v>
       </c>
       <c r="O193" t="n">
-        <v>1783294046793</v>
+        <v>1783298847047</v>
       </c>
       <c r="P193" t="inlineStr"/>
       <c r="Q193" s="2" t="n">
-        <v>46208.9773934375</v>
+        <v>46209.03295193287</v>
       </c>
       <c r="R193" t="n">
         <v>22.22</v>

</xml_diff>